<commit_message>
sync from erp-mapper@a36cff2: Merge feat/cleanup-A-cap-and-umbrella-titles — title simplification across 10 modules
</commit_message>
<xml_diff>
--- a/erp_checklist_type2.xlsx
+++ b/erp_checklist_type2.xlsx
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Financial Analytics &amp; Dashboards</t>
+          <t>Financial Analytics</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Tax Management &amp; GST Compliance</t>
+          <t>Tax Management</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Purchase Orders &amp; Procurement (Finance Side)</t>
+          <t>Purchase Orders (Finance Side)</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -3481,7 +3481,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Employee Master Record &amp; HRIS Core</t>
+          <t>Employee Master &amp; HRIS</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Leave &amp; Time-Off Management</t>
+          <t>Leave Management</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -3553,7 +3553,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Payroll Processing &amp; CPF Compliance</t>
+          <t>Payroll Processing</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Payslip Generation &amp; Distribution</t>
+          <t>Payslip Generation</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Onboarding &amp; Offboarding Workflows</t>
+          <t>Onboarding &amp; Offboarding</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Employee Self-Service Portal</t>
+          <t>Self-Service Portal</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Recruitment &amp; Applicant Tracking (ATS)</t>
+          <t>Recruitment &amp; ATS</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Performance Management &amp; Appraisals</t>
+          <t>Performance Management</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Compensation &amp; Benefits Management</t>
+          <t>Compensation Management</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Statutory HR Reporting (CPF, IRAS, MOM)</t>
+          <t>Statutory Reporting (CPF/IRAS/MOM)</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -3793,7 +3793,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Overtime &amp; Variable Pay Calculation</t>
+          <t>Overtime &amp; Variable Pay</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Organisation Chart &amp; Reporting Hierarchy</t>
+          <t>Organisation Chart</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Learning, Development &amp; Training Records</t>
+          <t>Learning &amp; Development</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Employee Engagement &amp; Surveys</t>
+          <t>Engagement &amp; Surveys</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Employee Expense &amp; Claims</t>
+          <t>Expense &amp; Claims</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Workforce Planning &amp; Headcount Forecasting</t>
+          <t>Workforce Planning</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Shift Scheduling &amp; Roster Management</t>
+          <t>Shift &amp; Roster Scheduling</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Work Permit &amp; Foreign Worker Management</t>
+          <t>Work Permit Management</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Time-Off Balance &amp; Accrual Engine</t>
+          <t>Time-Off Accrual Engine</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Disciplinary &amp; Grievance Management</t>
+          <t>Disciplinary &amp; Grievance</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -4047,7 +4047,7 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Exit Interviews &amp; Alumni Management</t>
+          <t>Exit &amp; Alumni</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>HR Analytics &amp; Dashboards</t>
+          <t>HR Analytics</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Employee Rewards &amp; Recognition</t>
+          <t>Rewards &amp; Recognition</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Marketing Website, CMS &amp; SEO Tools</t>
+          <t>Marketing Website &amp; SEO</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Partner Relationship Management (PRM)</t>
+          <t>Partner Relationship Management</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Social Engagement &amp; Inbox (Basic)</t>
+          <t>Social Engagement (Basic)</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -4790,7 +4790,7 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Customer Journey Orchestration &amp; Lifecycle Automation</t>
+          <t>Customer Journey Orchestration</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Subscription &amp; Recurring Revenue Management</t>
+          <t>Subscription Management</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Contract Tracking &amp; E-Signature (Basic)</t>
+          <t>Contract Tracking (Basic)</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Sales Enablement &amp; Content Management</t>
+          <t>Sales Enablement</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Voice of Customer, Surveys &amp; NPS</t>
+          <t>Voice of Customer &amp; NPS</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Omnichannel Retail (Basic — Physical+Digital)</t>
+          <t>Omnichannel Retail (Basic)</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Telephony, VoIP &amp; Communication Integration</t>
+          <t>Telephony &amp; VoIP Integration</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Inventory Master &amp; Item Management</t>
+          <t>Item Master Management</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -5233,7 +5233,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Stock Levels &amp; Warehouse Management</t>
+          <t>Stock Levels &amp; Warehouse</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Supply Chain Analytics &amp; Dashboards</t>
+          <t>Supply Chain Analytics</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -5511,7 +5511,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Multi-Warehouse &amp; Multi-Location Management</t>
+          <t>Multi-Warehouse Management</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Lot &amp; Serial Number Tracking</t>
+          <t>Lot &amp; Serial Tracking</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Kit, Bundle &amp; Assembly Management</t>
+          <t>Kit &amp; Bundle Management</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Quality Inspection &amp; Control</t>
+          <t>Quality Control</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Procurement Analytics &amp; Spend Analysis</t>
+          <t>Procurement Analytics</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Import/Export &amp; Trade Compliance</t>
+          <t>Trade Compliance</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -6027,7 +6027,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Bill of Materials (BOM)</t>
+          <t>Bill of Materials</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Material Requirements Planning (MRP)</t>
+          <t>Material Requirements Planning</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -6147,7 +6147,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Quality Management (QM)</t>
+          <t>Quality Management</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Manufacturing Safety, EHS &amp; Regulatory Compliance</t>
+          <t>Manufacturing EHS Compliance</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -6281,7 +6281,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Shop Floor Execution &amp; MES</t>
+          <t>Shop Floor Execution</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Engineering Change Management (ECO / ECR)</t>
+          <t>Engineering Change Management</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Product Master &amp; Document Management (Basic)</t>
+          <t>Product Master (Basic)</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -6397,7 +6397,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Mixed-Mode &amp; Configure-to-Order Manufacturing</t>
+          <t>Configure-to-Order Manufacturing</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -6469,7 +6469,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>IoT, Machine Integration &amp; Data Collection</t>
+          <t>IoT &amp; Machine Data Collection</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -6493,7 +6493,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>OEE &amp; Manufacturing Performance Analytics</t>
+          <t>OEE &amp; Performance Analytics</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -6541,7 +6541,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Labour Tracking &amp; Shop Floor Time Management</t>
+          <t>Labour &amp; Shop Floor Time</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Maintenance Integration (CMMS / EAM Linkage)</t>
+          <t>Maintenance Integration</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -6985,7 +6985,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Maintenance Requests &amp; Service Desk</t>
+          <t>Maintenance Requests</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -7009,7 +7009,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Spare Parts &amp; Maintenance Inventory</t>
+          <t>Spare Parts Management</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Condition Monitoring &amp; Predictive Maintenance</t>
+          <t>Condition Monitoring</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -7143,7 +7143,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Warranty &amp; Service Contracts</t>
+          <t>Warranty &amp; Contracts</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Capital Projects &amp; New Asset Commissioning</t>
+          <t>Capital Projects &amp; Commissioning</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Geospatial Asset Visualisation &amp; GIS Integration</t>
+          <t>Geospatial &amp; GIS Integration</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -7215,7 +7215,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Asset SLA &amp; Commercial Uptime Management</t>
+          <t>Asset SLA Management</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -7239,7 +7239,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Energy &amp; Carbon Tracking per Asset</t>
+          <t>Energy &amp; Carbon per Asset</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Disconnected / Offline Field Operations</t>
+          <t>Offline Field Operations</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Asset Leasing &amp; Lease Accounting</t>
+          <t>Asset Leasing</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">

</xml_diff>